<commit_message>
Planilla de multas: filas más altas en Administración para ver el relato y recálculo al abrir
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BuuNBJNJhyeT8FSxY2rfRA
</commit_message>
<xml_diff>
--- a/multas/Registro_Multas_Propietarios.xlsx
+++ b/multas/Registro_Multas_Propietarios.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="53">
   <si>
     <t xml:space="preserve">CÓMO SE USA</t>
   </si>
@@ -53,6 +53,9 @@
     <t xml:space="preserve">6. IMPORTANTE: no borrar ni ordenar filas en 'Carga Vigilador'; si un acta se anula, escribirlo en Observaciones.</t>
   </si>
   <si>
+    <t xml:space="preserve">6b. Si un relato es muy largo y no entra en la celda de Administración, hacer clic en la celda: el texto completo aparece en la barra de fórmulas.</t>
+  </si>
+  <si>
     <t xml:space="preserve">7. La fila 4 tiene de ejemplo el acta del 13/10/2026 (lote 92). Reemplazar el nombre del vigilador.</t>
   </si>
   <si>
@@ -60,6 +63,9 @@
   </si>
   <si>
     <t xml:space="preserve">Subir el archivo → Abrir con Hojas de cálculo de Google → Archivo → Guardar como Hojas de cálculo de Google.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OJO: la vista previa de Drive (sin convertir) NO actualiza las fórmulas; hay que trabajar sobre la versión convertida a Hojas de cálculo de Google.</t>
   </si>
   <si>
     <t xml:space="preserve">Recomendado: Datos → Proteger hojas y rangos, para que la guardia solo edite 'Carga Vigilador' y la administración 'Carga Administración'.</t>
@@ -833,7 +839,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="105"/>
@@ -888,21 +894,31 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="2"/>
-    </row>
-    <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="1" t="s">
+      <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="2"/>
+    </row>
+    <row r="13" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -935,35 +951,35 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -978,16 +994,16 @@
         <v>0.534027777777778</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E4" s="10" t="n">
         <v>92</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7011,7 +7027,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="70"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="10"/>
@@ -7023,56 +7039,56 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7115,7 +7131,7 @@
         <v>Pendiente</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A5="","",'Carga Vigilador'!A5)</f>
         <v/>
@@ -7155,7 +7171,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A6="","",'Carga Vigilador'!A6)</f>
         <v/>
@@ -7195,7 +7211,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A7="","",'Carga Vigilador'!A7)</f>
         <v/>
@@ -7235,7 +7251,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A8="","",'Carga Vigilador'!A8)</f>
         <v/>
@@ -7275,7 +7291,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A9="","",'Carga Vigilador'!A9)</f>
         <v/>
@@ -7315,7 +7331,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A10="","",'Carga Vigilador'!A10)</f>
         <v/>
@@ -7355,7 +7371,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A11="","",'Carga Vigilador'!A11)</f>
         <v/>
@@ -7395,7 +7411,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A12="","",'Carga Vigilador'!A12)</f>
         <v/>
@@ -7435,7 +7451,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A13="","",'Carga Vigilador'!A13)</f>
         <v/>
@@ -7475,7 +7491,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A14="","",'Carga Vigilador'!A14)</f>
         <v/>
@@ -7515,7 +7531,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A15="","",'Carga Vigilador'!A15)</f>
         <v/>
@@ -7555,7 +7571,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A16="","",'Carga Vigilador'!A16)</f>
         <v/>
@@ -7595,7 +7611,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A17="","",'Carga Vigilador'!A17)</f>
         <v/>
@@ -7635,7 +7651,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A18="","",'Carga Vigilador'!A18)</f>
         <v/>
@@ -7675,7 +7691,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A19="","",'Carga Vigilador'!A19)</f>
         <v/>
@@ -7715,7 +7731,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A20="","",'Carga Vigilador'!A20)</f>
         <v/>
@@ -7755,7 +7771,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A21="","",'Carga Vigilador'!A21)</f>
         <v/>
@@ -7795,7 +7811,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A22="","",'Carga Vigilador'!A22)</f>
         <v/>
@@ -7835,7 +7851,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A23="","",'Carga Vigilador'!A23)</f>
         <v/>
@@ -7875,7 +7891,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A24="","",'Carga Vigilador'!A24)</f>
         <v/>
@@ -7915,7 +7931,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A25="","",'Carga Vigilador'!A25)</f>
         <v/>
@@ -7955,7 +7971,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A26="","",'Carga Vigilador'!A26)</f>
         <v/>
@@ -7995,7 +8011,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A27="","",'Carga Vigilador'!A27)</f>
         <v/>
@@ -8035,7 +8051,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A28="","",'Carga Vigilador'!A28)</f>
         <v/>
@@ -8075,7 +8091,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A29="","",'Carga Vigilador'!A29)</f>
         <v/>
@@ -8115,7 +8131,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A30="","",'Carga Vigilador'!A30)</f>
         <v/>
@@ -8155,7 +8171,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A31="","",'Carga Vigilador'!A31)</f>
         <v/>
@@ -8195,7 +8211,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A32="","",'Carga Vigilador'!A32)</f>
         <v/>
@@ -8235,7 +8251,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A33="","",'Carga Vigilador'!A33)</f>
         <v/>
@@ -8275,7 +8291,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A34="","",'Carga Vigilador'!A34)</f>
         <v/>
@@ -8315,7 +8331,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A35="","",'Carga Vigilador'!A35)</f>
         <v/>
@@ -8355,7 +8371,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A36="","",'Carga Vigilador'!A36)</f>
         <v/>
@@ -8395,7 +8411,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A37="","",'Carga Vigilador'!A37)</f>
         <v/>
@@ -8435,7 +8451,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A38="","",'Carga Vigilador'!A38)</f>
         <v/>
@@ -8475,7 +8491,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A39="","",'Carga Vigilador'!A39)</f>
         <v/>
@@ -8515,7 +8531,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A40="","",'Carga Vigilador'!A40)</f>
         <v/>
@@ -8555,7 +8571,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A41="","",'Carga Vigilador'!A41)</f>
         <v/>
@@ -8595,7 +8611,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A42="","",'Carga Vigilador'!A42)</f>
         <v/>
@@ -8635,7 +8651,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A43="","",'Carga Vigilador'!A43)</f>
         <v/>
@@ -8675,7 +8691,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A44="","",'Carga Vigilador'!A44)</f>
         <v/>
@@ -8715,7 +8731,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A45="","",'Carga Vigilador'!A45)</f>
         <v/>
@@ -8755,7 +8771,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A46="","",'Carga Vigilador'!A46)</f>
         <v/>
@@ -8795,7 +8811,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A47="","",'Carga Vigilador'!A47)</f>
         <v/>
@@ -8835,7 +8851,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A48="","",'Carga Vigilador'!A48)</f>
         <v/>
@@ -8875,7 +8891,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A49="","",'Carga Vigilador'!A49)</f>
         <v/>
@@ -8915,7 +8931,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A50="","",'Carga Vigilador'!A50)</f>
         <v/>
@@ -8955,7 +8971,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A51="","",'Carga Vigilador'!A51)</f>
         <v/>
@@ -8995,7 +9011,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A52="","",'Carga Vigilador'!A52)</f>
         <v/>
@@ -9035,7 +9051,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A53="","",'Carga Vigilador'!A53)</f>
         <v/>
@@ -9075,7 +9091,7 @@
         <v/>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A54="","",'Carga Vigilador'!A54)</f>
         <v/>
@@ -9115,7 +9131,7 @@
         <v/>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A55="","",'Carga Vigilador'!A55)</f>
         <v/>
@@ -9155,7 +9171,7 @@
         <v/>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A56="","",'Carga Vigilador'!A56)</f>
         <v/>
@@ -9195,7 +9211,7 @@
         <v/>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A57="","",'Carga Vigilador'!A57)</f>
         <v/>
@@ -9235,7 +9251,7 @@
         <v/>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A58="","",'Carga Vigilador'!A58)</f>
         <v/>
@@ -9275,7 +9291,7 @@
         <v/>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A59="","",'Carga Vigilador'!A59)</f>
         <v/>
@@ -9315,7 +9331,7 @@
         <v/>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A60="","",'Carga Vigilador'!A60)</f>
         <v/>
@@ -9355,7 +9371,7 @@
         <v/>
       </c>
     </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A61="","",'Carga Vigilador'!A61)</f>
         <v/>
@@ -9395,7 +9411,7 @@
         <v/>
       </c>
     </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A62="","",'Carga Vigilador'!A62)</f>
         <v/>
@@ -9435,7 +9451,7 @@
         <v/>
       </c>
     </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A63="","",'Carga Vigilador'!A63)</f>
         <v/>
@@ -9475,7 +9491,7 @@
         <v/>
       </c>
     </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A64="","",'Carga Vigilador'!A64)</f>
         <v/>
@@ -9515,7 +9531,7 @@
         <v/>
       </c>
     </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A65="","",'Carga Vigilador'!A65)</f>
         <v/>
@@ -9555,7 +9571,7 @@
         <v/>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A66="","",'Carga Vigilador'!A66)</f>
         <v/>
@@ -9595,7 +9611,7 @@
         <v/>
       </c>
     </row>
-    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="67" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A67="","",'Carga Vigilador'!A67)</f>
         <v/>
@@ -9635,7 +9651,7 @@
         <v/>
       </c>
     </row>
-    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="68" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A68="","",'Carga Vigilador'!A68)</f>
         <v/>
@@ -9675,7 +9691,7 @@
         <v/>
       </c>
     </row>
-    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="69" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A69="","",'Carga Vigilador'!A69)</f>
         <v/>
@@ -9715,7 +9731,7 @@
         <v/>
       </c>
     </row>
-    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="70" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A70="","",'Carga Vigilador'!A70)</f>
         <v/>
@@ -9755,7 +9771,7 @@
         <v/>
       </c>
     </row>
-    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="71" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A71="","",'Carga Vigilador'!A71)</f>
         <v/>
@@ -9795,7 +9811,7 @@
         <v/>
       </c>
     </row>
-    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="72" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A72="","",'Carga Vigilador'!A72)</f>
         <v/>
@@ -9835,7 +9851,7 @@
         <v/>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A73="","",'Carga Vigilador'!A73)</f>
         <v/>
@@ -9875,7 +9891,7 @@
         <v/>
       </c>
     </row>
-    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="74" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A74="","",'Carga Vigilador'!A74)</f>
         <v/>
@@ -9915,7 +9931,7 @@
         <v/>
       </c>
     </row>
-    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="75" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A75="","",'Carga Vigilador'!A75)</f>
         <v/>
@@ -9955,7 +9971,7 @@
         <v/>
       </c>
     </row>
-    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="76" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A76="","",'Carga Vigilador'!A76)</f>
         <v/>
@@ -9995,7 +10011,7 @@
         <v/>
       </c>
     </row>
-    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="77" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A77="","",'Carga Vigilador'!A77)</f>
         <v/>
@@ -10035,7 +10051,7 @@
         <v/>
       </c>
     </row>
-    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="78" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A78="","",'Carga Vigilador'!A78)</f>
         <v/>
@@ -10075,7 +10091,7 @@
         <v/>
       </c>
     </row>
-    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="79" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A79="","",'Carga Vigilador'!A79)</f>
         <v/>
@@ -10115,7 +10131,7 @@
         <v/>
       </c>
     </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="80" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A80="","",'Carga Vigilador'!A80)</f>
         <v/>
@@ -10155,7 +10171,7 @@
         <v/>
       </c>
     </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="81" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A81="","",'Carga Vigilador'!A81)</f>
         <v/>
@@ -10195,7 +10211,7 @@
         <v/>
       </c>
     </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="82" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A82="","",'Carga Vigilador'!A82)</f>
         <v/>
@@ -10235,7 +10251,7 @@
         <v/>
       </c>
     </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="83" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A83="","",'Carga Vigilador'!A83)</f>
         <v/>
@@ -10275,7 +10291,7 @@
         <v/>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A84="","",'Carga Vigilador'!A84)</f>
         <v/>
@@ -10315,7 +10331,7 @@
         <v/>
       </c>
     </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="85" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A85="","",'Carga Vigilador'!A85)</f>
         <v/>
@@ -10355,7 +10371,7 @@
         <v/>
       </c>
     </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="86" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A86="","",'Carga Vigilador'!A86)</f>
         <v/>
@@ -10395,7 +10411,7 @@
         <v/>
       </c>
     </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="87" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A87="","",'Carga Vigilador'!A87)</f>
         <v/>
@@ -10435,7 +10451,7 @@
         <v/>
       </c>
     </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="88" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A88="","",'Carga Vigilador'!A88)</f>
         <v/>
@@ -10475,7 +10491,7 @@
         <v/>
       </c>
     </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="89" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A89="","",'Carga Vigilador'!A89)</f>
         <v/>
@@ -10515,7 +10531,7 @@
         <v/>
       </c>
     </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="90" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A90="","",'Carga Vigilador'!A90)</f>
         <v/>
@@ -10555,7 +10571,7 @@
         <v/>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A91="","",'Carga Vigilador'!A91)</f>
         <v/>
@@ -10595,7 +10611,7 @@
         <v/>
       </c>
     </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="92" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A92="","",'Carga Vigilador'!A92)</f>
         <v/>
@@ -10635,7 +10651,7 @@
         <v/>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A93="","",'Carga Vigilador'!A93)</f>
         <v/>
@@ -10675,7 +10691,7 @@
         <v/>
       </c>
     </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="94" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A94="","",'Carga Vigilador'!A94)</f>
         <v/>
@@ -10715,7 +10731,7 @@
         <v/>
       </c>
     </row>
-    <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="95" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A95="","",'Carga Vigilador'!A95)</f>
         <v/>
@@ -10755,7 +10771,7 @@
         <v/>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A96="","",'Carga Vigilador'!A96)</f>
         <v/>
@@ -10795,7 +10811,7 @@
         <v/>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A97="","",'Carga Vigilador'!A97)</f>
         <v/>
@@ -10835,7 +10851,7 @@
         <v/>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A98="","",'Carga Vigilador'!A98)</f>
         <v/>
@@ -10875,7 +10891,7 @@
         <v/>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A99="","",'Carga Vigilador'!A99)</f>
         <v/>
@@ -10915,7 +10931,7 @@
         <v/>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A100="","",'Carga Vigilador'!A100)</f>
         <v/>
@@ -10955,7 +10971,7 @@
         <v/>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A101="","",'Carga Vigilador'!A101)</f>
         <v/>
@@ -10995,7 +11011,7 @@
         <v/>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A102="","",'Carga Vigilador'!A102)</f>
         <v/>
@@ -11035,7 +11051,7 @@
         <v/>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A103="","",'Carga Vigilador'!A103)</f>
         <v/>
@@ -11075,7 +11091,7 @@
         <v/>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A104="","",'Carga Vigilador'!A104)</f>
         <v/>
@@ -11115,7 +11131,7 @@
         <v/>
       </c>
     </row>
-    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="105" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A105="","",'Carga Vigilador'!A105)</f>
         <v/>
@@ -11155,7 +11171,7 @@
         <v/>
       </c>
     </row>
-    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="106" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A106="","",'Carga Vigilador'!A106)</f>
         <v/>
@@ -11195,7 +11211,7 @@
         <v/>
       </c>
     </row>
-    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="107" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A107="","",'Carga Vigilador'!A107)</f>
         <v/>
@@ -11235,7 +11251,7 @@
         <v/>
       </c>
     </row>
-    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="108" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A108="","",'Carga Vigilador'!A108)</f>
         <v/>
@@ -11275,7 +11291,7 @@
         <v/>
       </c>
     </row>
-    <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="109" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A109="","",'Carga Vigilador'!A109)</f>
         <v/>
@@ -11315,7 +11331,7 @@
         <v/>
       </c>
     </row>
-    <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="110" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A110="","",'Carga Vigilador'!A110)</f>
         <v/>
@@ -11355,7 +11371,7 @@
         <v/>
       </c>
     </row>
-    <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="111" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A111="","",'Carga Vigilador'!A111)</f>
         <v/>
@@ -11395,7 +11411,7 @@
         <v/>
       </c>
     </row>
-    <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="112" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A112="","",'Carga Vigilador'!A112)</f>
         <v/>
@@ -11435,7 +11451,7 @@
         <v/>
       </c>
     </row>
-    <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="113" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A113="","",'Carga Vigilador'!A113)</f>
         <v/>
@@ -11475,7 +11491,7 @@
         <v/>
       </c>
     </row>
-    <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A114="","",'Carga Vigilador'!A114)</f>
         <v/>
@@ -11515,7 +11531,7 @@
         <v/>
       </c>
     </row>
-    <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="115" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A115="","",'Carga Vigilador'!A115)</f>
         <v/>
@@ -11555,7 +11571,7 @@
         <v/>
       </c>
     </row>
-    <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A116="","",'Carga Vigilador'!A116)</f>
         <v/>
@@ -11595,7 +11611,7 @@
         <v/>
       </c>
     </row>
-    <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A117="","",'Carga Vigilador'!A117)</f>
         <v/>
@@ -11635,7 +11651,7 @@
         <v/>
       </c>
     </row>
-    <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="118" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A118="","",'Carga Vigilador'!A118)</f>
         <v/>
@@ -11675,7 +11691,7 @@
         <v/>
       </c>
     </row>
-    <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A119="","",'Carga Vigilador'!A119)</f>
         <v/>
@@ -11715,7 +11731,7 @@
         <v/>
       </c>
     </row>
-    <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A120="","",'Carga Vigilador'!A120)</f>
         <v/>
@@ -11755,7 +11771,7 @@
         <v/>
       </c>
     </row>
-    <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="121" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A121="","",'Carga Vigilador'!A121)</f>
         <v/>
@@ -11795,7 +11811,7 @@
         <v/>
       </c>
     </row>
-    <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="122" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A122="","",'Carga Vigilador'!A122)</f>
         <v/>
@@ -11835,7 +11851,7 @@
         <v/>
       </c>
     </row>
-    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A123="","",'Carga Vigilador'!A123)</f>
         <v/>
@@ -11875,7 +11891,7 @@
         <v/>
       </c>
     </row>
-    <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A124="","",'Carga Vigilador'!A124)</f>
         <v/>
@@ -11915,7 +11931,7 @@
         <v/>
       </c>
     </row>
-    <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A125="","",'Carga Vigilador'!A125)</f>
         <v/>
@@ -11955,7 +11971,7 @@
         <v/>
       </c>
     </row>
-    <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A126="","",'Carga Vigilador'!A126)</f>
         <v/>
@@ -11995,7 +12011,7 @@
         <v/>
       </c>
     </row>
-    <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="127" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A127="","",'Carga Vigilador'!A127)</f>
         <v/>
@@ -12035,7 +12051,7 @@
         <v/>
       </c>
     </row>
-    <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A128="","",'Carga Vigilador'!A128)</f>
         <v/>
@@ -12075,7 +12091,7 @@
         <v/>
       </c>
     </row>
-    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A129="","",'Carga Vigilador'!A129)</f>
         <v/>
@@ -12115,7 +12131,7 @@
         <v/>
       </c>
     </row>
-    <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A130="","",'Carga Vigilador'!A130)</f>
         <v/>
@@ -12155,7 +12171,7 @@
         <v/>
       </c>
     </row>
-    <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="131" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A131="","",'Carga Vigilador'!A131)</f>
         <v/>
@@ -12195,7 +12211,7 @@
         <v/>
       </c>
     </row>
-    <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="132" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A132="","",'Carga Vigilador'!A132)</f>
         <v/>
@@ -12235,7 +12251,7 @@
         <v/>
       </c>
     </row>
-    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A133="","",'Carga Vigilador'!A133)</f>
         <v/>
@@ -12275,7 +12291,7 @@
         <v/>
       </c>
     </row>
-    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A134="","",'Carga Vigilador'!A134)</f>
         <v/>
@@ -12315,7 +12331,7 @@
         <v/>
       </c>
     </row>
-    <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A135="","",'Carga Vigilador'!A135)</f>
         <v/>
@@ -12355,7 +12371,7 @@
         <v/>
       </c>
     </row>
-    <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="136" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A136="","",'Carga Vigilador'!A136)</f>
         <v/>
@@ -12395,7 +12411,7 @@
         <v/>
       </c>
     </row>
-    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="137" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A137="","",'Carga Vigilador'!A137)</f>
         <v/>
@@ -12435,7 +12451,7 @@
         <v/>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A138="","",'Carga Vigilador'!A138)</f>
         <v/>
@@ -12475,7 +12491,7 @@
         <v/>
       </c>
     </row>
-    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A139="","",'Carga Vigilador'!A139)</f>
         <v/>
@@ -12515,7 +12531,7 @@
         <v/>
       </c>
     </row>
-    <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="140" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A140="","",'Carga Vigilador'!A140)</f>
         <v/>
@@ -12555,7 +12571,7 @@
         <v/>
       </c>
     </row>
-    <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A141="","",'Carga Vigilador'!A141)</f>
         <v/>
@@ -12595,7 +12611,7 @@
         <v/>
       </c>
     </row>
-    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="142" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A142="","",'Carga Vigilador'!A142)</f>
         <v/>
@@ -12635,7 +12651,7 @@
         <v/>
       </c>
     </row>
-    <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="143" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A143="","",'Carga Vigilador'!A143)</f>
         <v/>
@@ -12675,7 +12691,7 @@
         <v/>
       </c>
     </row>
-    <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A144="","",'Carga Vigilador'!A144)</f>
         <v/>
@@ -12715,7 +12731,7 @@
         <v/>
       </c>
     </row>
-    <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="145" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A145="","",'Carga Vigilador'!A145)</f>
         <v/>
@@ -12755,7 +12771,7 @@
         <v/>
       </c>
     </row>
-    <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="146" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A146="","",'Carga Vigilador'!A146)</f>
         <v/>
@@ -12795,7 +12811,7 @@
         <v/>
       </c>
     </row>
-    <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="147" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A147="","",'Carga Vigilador'!A147)</f>
         <v/>
@@ -12835,7 +12851,7 @@
         <v/>
       </c>
     </row>
-    <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="148" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A148="","",'Carga Vigilador'!A148)</f>
         <v/>
@@ -12875,7 +12891,7 @@
         <v/>
       </c>
     </row>
-    <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="149" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A149="","",'Carga Vigilador'!A149)</f>
         <v/>
@@ -12915,7 +12931,7 @@
         <v/>
       </c>
     </row>
-    <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="150" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A150="","",'Carga Vigilador'!A150)</f>
         <v/>
@@ -12955,7 +12971,7 @@
         <v/>
       </c>
     </row>
-    <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="151" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A151="","",'Carga Vigilador'!A151)</f>
         <v/>
@@ -12995,7 +13011,7 @@
         <v/>
       </c>
     </row>
-    <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="152" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A152="","",'Carga Vigilador'!A152)</f>
         <v/>
@@ -13035,7 +13051,7 @@
         <v/>
       </c>
     </row>
-    <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="153" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A153="","",'Carga Vigilador'!A153)</f>
         <v/>
@@ -13075,7 +13091,7 @@
         <v/>
       </c>
     </row>
-    <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="154" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A154="","",'Carga Vigilador'!A154)</f>
         <v/>
@@ -13115,7 +13131,7 @@
         <v/>
       </c>
     </row>
-    <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="155" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A155="","",'Carga Vigilador'!A155)</f>
         <v/>
@@ -13155,7 +13171,7 @@
         <v/>
       </c>
     </row>
-    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="156" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A156="","",'Carga Vigilador'!A156)</f>
         <v/>
@@ -13195,7 +13211,7 @@
         <v/>
       </c>
     </row>
-    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="157" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A157="","",'Carga Vigilador'!A157)</f>
         <v/>
@@ -13235,7 +13251,7 @@
         <v/>
       </c>
     </row>
-    <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="158" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A158="","",'Carga Vigilador'!A158)</f>
         <v/>
@@ -13275,7 +13291,7 @@
         <v/>
       </c>
     </row>
-    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="159" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A159="","",'Carga Vigilador'!A159)</f>
         <v/>
@@ -13315,7 +13331,7 @@
         <v/>
       </c>
     </row>
-    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="160" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A160="","",'Carga Vigilador'!A160)</f>
         <v/>
@@ -13355,7 +13371,7 @@
         <v/>
       </c>
     </row>
-    <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="161" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A161="","",'Carga Vigilador'!A161)</f>
         <v/>
@@ -13395,7 +13411,7 @@
         <v/>
       </c>
     </row>
-    <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="162" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A162="","",'Carga Vigilador'!A162)</f>
         <v/>
@@ -13435,7 +13451,7 @@
         <v/>
       </c>
     </row>
-    <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="163" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A163="","",'Carga Vigilador'!A163)</f>
         <v/>
@@ -13475,7 +13491,7 @@
         <v/>
       </c>
     </row>
-    <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="164" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A164="","",'Carga Vigilador'!A164)</f>
         <v/>
@@ -13515,7 +13531,7 @@
         <v/>
       </c>
     </row>
-    <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="165" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A165="","",'Carga Vigilador'!A165)</f>
         <v/>
@@ -13555,7 +13571,7 @@
         <v/>
       </c>
     </row>
-    <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="166" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A166="","",'Carga Vigilador'!A166)</f>
         <v/>
@@ -13595,7 +13611,7 @@
         <v/>
       </c>
     </row>
-    <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="167" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A167="","",'Carga Vigilador'!A167)</f>
         <v/>
@@ -13635,7 +13651,7 @@
         <v/>
       </c>
     </row>
-    <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="168" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A168="","",'Carga Vigilador'!A168)</f>
         <v/>
@@ -13675,7 +13691,7 @@
         <v/>
       </c>
     </row>
-    <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="169" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A169="","",'Carga Vigilador'!A169)</f>
         <v/>
@@ -13715,7 +13731,7 @@
         <v/>
       </c>
     </row>
-    <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="170" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A170="","",'Carga Vigilador'!A170)</f>
         <v/>
@@ -13755,7 +13771,7 @@
         <v/>
       </c>
     </row>
-    <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="171" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A171="","",'Carga Vigilador'!A171)</f>
         <v/>
@@ -13795,7 +13811,7 @@
         <v/>
       </c>
     </row>
-    <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="172" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A172="","",'Carga Vigilador'!A172)</f>
         <v/>
@@ -13835,7 +13851,7 @@
         <v/>
       </c>
     </row>
-    <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="173" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A173="","",'Carga Vigilador'!A173)</f>
         <v/>
@@ -13875,7 +13891,7 @@
         <v/>
       </c>
     </row>
-    <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="174" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A174="","",'Carga Vigilador'!A174)</f>
         <v/>
@@ -13915,7 +13931,7 @@
         <v/>
       </c>
     </row>
-    <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="175" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A175="","",'Carga Vigilador'!A175)</f>
         <v/>
@@ -13955,7 +13971,7 @@
         <v/>
       </c>
     </row>
-    <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="176" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A176="","",'Carga Vigilador'!A176)</f>
         <v/>
@@ -13995,7 +14011,7 @@
         <v/>
       </c>
     </row>
-    <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="177" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A177="","",'Carga Vigilador'!A177)</f>
         <v/>
@@ -14035,7 +14051,7 @@
         <v/>
       </c>
     </row>
-    <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="178" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A178="","",'Carga Vigilador'!A178)</f>
         <v/>
@@ -14075,7 +14091,7 @@
         <v/>
       </c>
     </row>
-    <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="179" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A179="","",'Carga Vigilador'!A179)</f>
         <v/>
@@ -14115,7 +14131,7 @@
         <v/>
       </c>
     </row>
-    <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="180" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A180="","",'Carga Vigilador'!A180)</f>
         <v/>
@@ -14155,7 +14171,7 @@
         <v/>
       </c>
     </row>
-    <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="181" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A181="","",'Carga Vigilador'!A181)</f>
         <v/>
@@ -14195,7 +14211,7 @@
         <v/>
       </c>
     </row>
-    <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="182" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A182" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A182="","",'Carga Vigilador'!A182)</f>
         <v/>
@@ -14235,7 +14251,7 @@
         <v/>
       </c>
     </row>
-    <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="183" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A183" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A183="","",'Carga Vigilador'!A183)</f>
         <v/>
@@ -14275,7 +14291,7 @@
         <v/>
       </c>
     </row>
-    <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="184" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A184" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A184="","",'Carga Vigilador'!A184)</f>
         <v/>
@@ -14315,7 +14331,7 @@
         <v/>
       </c>
     </row>
-    <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="185" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A185" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A185="","",'Carga Vigilador'!A185)</f>
         <v/>
@@ -14355,7 +14371,7 @@
         <v/>
       </c>
     </row>
-    <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="186" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A186" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A186="","",'Carga Vigilador'!A186)</f>
         <v/>
@@ -14395,7 +14411,7 @@
         <v/>
       </c>
     </row>
-    <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="187" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A187" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A187="","",'Carga Vigilador'!A187)</f>
         <v/>
@@ -14435,7 +14451,7 @@
         <v/>
       </c>
     </row>
-    <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="188" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A188" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A188="","",'Carga Vigilador'!A188)</f>
         <v/>
@@ -14475,7 +14491,7 @@
         <v/>
       </c>
     </row>
-    <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="189" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A189" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A189="","",'Carga Vigilador'!A189)</f>
         <v/>
@@ -14515,7 +14531,7 @@
         <v/>
       </c>
     </row>
-    <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="190" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A190" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A190="","",'Carga Vigilador'!A190)</f>
         <v/>
@@ -14555,7 +14571,7 @@
         <v/>
       </c>
     </row>
-    <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="191" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A191" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A191="","",'Carga Vigilador'!A191)</f>
         <v/>
@@ -14595,7 +14611,7 @@
         <v/>
       </c>
     </row>
-    <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="192" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A192" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A192="","",'Carga Vigilador'!A192)</f>
         <v/>
@@ -14635,7 +14651,7 @@
         <v/>
       </c>
     </row>
-    <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="193" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A193" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A193="","",'Carga Vigilador'!A193)</f>
         <v/>
@@ -14675,7 +14691,7 @@
         <v/>
       </c>
     </row>
-    <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="194" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A194" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A194="","",'Carga Vigilador'!A194)</f>
         <v/>
@@ -14715,7 +14731,7 @@
         <v/>
       </c>
     </row>
-    <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="195" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A195" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A195="","",'Carga Vigilador'!A195)</f>
         <v/>
@@ -14755,7 +14771,7 @@
         <v/>
       </c>
     </row>
-    <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="196" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A196" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A196="","",'Carga Vigilador'!A196)</f>
         <v/>
@@ -14795,7 +14811,7 @@
         <v/>
       </c>
     </row>
-    <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="197" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A197" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A197="","",'Carga Vigilador'!A197)</f>
         <v/>
@@ -14835,7 +14851,7 @@
         <v/>
       </c>
     </row>
-    <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="198" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A198" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A198="","",'Carga Vigilador'!A198)</f>
         <v/>
@@ -14875,7 +14891,7 @@
         <v/>
       </c>
     </row>
-    <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="199" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A199" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A199="","",'Carga Vigilador'!A199)</f>
         <v/>
@@ -14915,7 +14931,7 @@
         <v/>
       </c>
     </row>
-    <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="200" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A200" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A200="","",'Carga Vigilador'!A200)</f>
         <v/>
@@ -14955,7 +14971,7 @@
         <v/>
       </c>
     </row>
-    <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="201" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A201" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A201="","",'Carga Vigilador'!A201)</f>
         <v/>
@@ -14995,7 +15011,7 @@
         <v/>
       </c>
     </row>
-    <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="202" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A202" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A202="","",'Carga Vigilador'!A202)</f>
         <v/>
@@ -15035,7 +15051,7 @@
         <v/>
       </c>
     </row>
-    <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="203" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A203" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A203="","",'Carga Vigilador'!A203)</f>
         <v/>
@@ -15075,7 +15091,7 @@
         <v/>
       </c>
     </row>
-    <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="204" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A204" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A204="","",'Carga Vigilador'!A204)</f>
         <v/>
@@ -15115,7 +15131,7 @@
         <v/>
       </c>
     </row>
-    <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="205" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A205" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A205="","",'Carga Vigilador'!A205)</f>
         <v/>
@@ -15155,7 +15171,7 @@
         <v/>
       </c>
     </row>
-    <row r="206" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="206" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A206" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A206="","",'Carga Vigilador'!A206)</f>
         <v/>
@@ -15195,7 +15211,7 @@
         <v/>
       </c>
     </row>
-    <row r="207" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="207" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A207" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A207="","",'Carga Vigilador'!A207)</f>
         <v/>
@@ -15235,7 +15251,7 @@
         <v/>
       </c>
     </row>
-    <row r="208" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="208" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A208" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A208="","",'Carga Vigilador'!A208)</f>
         <v/>
@@ -15275,7 +15291,7 @@
         <v/>
       </c>
     </row>
-    <row r="209" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="209" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A209" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A209="","",'Carga Vigilador'!A209)</f>
         <v/>
@@ -15315,7 +15331,7 @@
         <v/>
       </c>
     </row>
-    <row r="210" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="210" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A210" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A210="","",'Carga Vigilador'!A210)</f>
         <v/>
@@ -15355,7 +15371,7 @@
         <v/>
       </c>
     </row>
-    <row r="211" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="211" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A211" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A211="","",'Carga Vigilador'!A211)</f>
         <v/>
@@ -15395,7 +15411,7 @@
         <v/>
       </c>
     </row>
-    <row r="212" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="212" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A212" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A212="","",'Carga Vigilador'!A212)</f>
         <v/>
@@ -15435,7 +15451,7 @@
         <v/>
       </c>
     </row>
-    <row r="213" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="213" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A213" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A213="","",'Carga Vigilador'!A213)</f>
         <v/>
@@ -15475,7 +15491,7 @@
         <v/>
       </c>
     </row>
-    <row r="214" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="214" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A214" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A214="","",'Carga Vigilador'!A214)</f>
         <v/>
@@ -15515,7 +15531,7 @@
         <v/>
       </c>
     </row>
-    <row r="215" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="215" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A215" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A215="","",'Carga Vigilador'!A215)</f>
         <v/>
@@ -15555,7 +15571,7 @@
         <v/>
       </c>
     </row>
-    <row r="216" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="216" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A216" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A216="","",'Carga Vigilador'!A216)</f>
         <v/>
@@ -15595,7 +15611,7 @@
         <v/>
       </c>
     </row>
-    <row r="217" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="217" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A217" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A217="","",'Carga Vigilador'!A217)</f>
         <v/>
@@ -15635,7 +15651,7 @@
         <v/>
       </c>
     </row>
-    <row r="218" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="218" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A218" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A218="","",'Carga Vigilador'!A218)</f>
         <v/>
@@ -15675,7 +15691,7 @@
         <v/>
       </c>
     </row>
-    <row r="219" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="219" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A219" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A219="","",'Carga Vigilador'!A219)</f>
         <v/>
@@ -15715,7 +15731,7 @@
         <v/>
       </c>
     </row>
-    <row r="220" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="220" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A220" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A220="","",'Carga Vigilador'!A220)</f>
         <v/>
@@ -15755,7 +15771,7 @@
         <v/>
       </c>
     </row>
-    <row r="221" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="221" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A221" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A221="","",'Carga Vigilador'!A221)</f>
         <v/>
@@ -15795,7 +15811,7 @@
         <v/>
       </c>
     </row>
-    <row r="222" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="222" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A222" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A222="","",'Carga Vigilador'!A222)</f>
         <v/>
@@ -15835,7 +15851,7 @@
         <v/>
       </c>
     </row>
-    <row r="223" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="223" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A223" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A223="","",'Carga Vigilador'!A223)</f>
         <v/>
@@ -15875,7 +15891,7 @@
         <v/>
       </c>
     </row>
-    <row r="224" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="224" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A224" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A224="","",'Carga Vigilador'!A224)</f>
         <v/>
@@ -15915,7 +15931,7 @@
         <v/>
       </c>
     </row>
-    <row r="225" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="225" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A225" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A225="","",'Carga Vigilador'!A225)</f>
         <v/>
@@ -15955,7 +15971,7 @@
         <v/>
       </c>
     </row>
-    <row r="226" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="226" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A226" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A226="","",'Carga Vigilador'!A226)</f>
         <v/>
@@ -15995,7 +16011,7 @@
         <v/>
       </c>
     </row>
-    <row r="227" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="227" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A227" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A227="","",'Carga Vigilador'!A227)</f>
         <v/>
@@ -16035,7 +16051,7 @@
         <v/>
       </c>
     </row>
-    <row r="228" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="228" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A228" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A228="","",'Carga Vigilador'!A228)</f>
         <v/>
@@ -16075,7 +16091,7 @@
         <v/>
       </c>
     </row>
-    <row r="229" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="229" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A229" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A229="","",'Carga Vigilador'!A229)</f>
         <v/>
@@ -16115,7 +16131,7 @@
         <v/>
       </c>
     </row>
-    <row r="230" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="230" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A230" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A230="","",'Carga Vigilador'!A230)</f>
         <v/>
@@ -16155,7 +16171,7 @@
         <v/>
       </c>
     </row>
-    <row r="231" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="231" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A231" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A231="","",'Carga Vigilador'!A231)</f>
         <v/>
@@ -16195,7 +16211,7 @@
         <v/>
       </c>
     </row>
-    <row r="232" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="232" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A232" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A232="","",'Carga Vigilador'!A232)</f>
         <v/>
@@ -16235,7 +16251,7 @@
         <v/>
       </c>
     </row>
-    <row r="233" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="233" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A233" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A233="","",'Carga Vigilador'!A233)</f>
         <v/>
@@ -16275,7 +16291,7 @@
         <v/>
       </c>
     </row>
-    <row r="234" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="234" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A234" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A234="","",'Carga Vigilador'!A234)</f>
         <v/>
@@ -16315,7 +16331,7 @@
         <v/>
       </c>
     </row>
-    <row r="235" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="235" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A235" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A235="","",'Carga Vigilador'!A235)</f>
         <v/>
@@ -16355,7 +16371,7 @@
         <v/>
       </c>
     </row>
-    <row r="236" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="236" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A236" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A236="","",'Carga Vigilador'!A236)</f>
         <v/>
@@ -16395,7 +16411,7 @@
         <v/>
       </c>
     </row>
-    <row r="237" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="237" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A237" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A237="","",'Carga Vigilador'!A237)</f>
         <v/>
@@ -16435,7 +16451,7 @@
         <v/>
       </c>
     </row>
-    <row r="238" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="238" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A238" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A238="","",'Carga Vigilador'!A238)</f>
         <v/>
@@ -16475,7 +16491,7 @@
         <v/>
       </c>
     </row>
-    <row r="239" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="239" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A239" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A239="","",'Carga Vigilador'!A239)</f>
         <v/>
@@ -16515,7 +16531,7 @@
         <v/>
       </c>
     </row>
-    <row r="240" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="240" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A240" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A240="","",'Carga Vigilador'!A240)</f>
         <v/>
@@ -16555,7 +16571,7 @@
         <v/>
       </c>
     </row>
-    <row r="241" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="241" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A241" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A241="","",'Carga Vigilador'!A241)</f>
         <v/>
@@ -16595,7 +16611,7 @@
         <v/>
       </c>
     </row>
-    <row r="242" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="242" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A242" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A242="","",'Carga Vigilador'!A242)</f>
         <v/>
@@ -16635,7 +16651,7 @@
         <v/>
       </c>
     </row>
-    <row r="243" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="243" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A243" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A243="","",'Carga Vigilador'!A243)</f>
         <v/>
@@ -16675,7 +16691,7 @@
         <v/>
       </c>
     </row>
-    <row r="244" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="244" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A244" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A244="","",'Carga Vigilador'!A244)</f>
         <v/>
@@ -16715,7 +16731,7 @@
         <v/>
       </c>
     </row>
-    <row r="245" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="245" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A245" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A245="","",'Carga Vigilador'!A245)</f>
         <v/>
@@ -16755,7 +16771,7 @@
         <v/>
       </c>
     </row>
-    <row r="246" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="246" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A246" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A246="","",'Carga Vigilador'!A246)</f>
         <v/>
@@ -16795,7 +16811,7 @@
         <v/>
       </c>
     </row>
-    <row r="247" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="247" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A247" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A247="","",'Carga Vigilador'!A247)</f>
         <v/>
@@ -16835,7 +16851,7 @@
         <v/>
       </c>
     </row>
-    <row r="248" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="248" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A248" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A248="","",'Carga Vigilador'!A248)</f>
         <v/>
@@ -16875,7 +16891,7 @@
         <v/>
       </c>
     </row>
-    <row r="249" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="249" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A249" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A249="","",'Carga Vigilador'!A249)</f>
         <v/>
@@ -16915,7 +16931,7 @@
         <v/>
       </c>
     </row>
-    <row r="250" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="250" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A250" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A250="","",'Carga Vigilador'!A250)</f>
         <v/>
@@ -16955,7 +16971,7 @@
         <v/>
       </c>
     </row>
-    <row r="251" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="251" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A251" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A251="","",'Carga Vigilador'!A251)</f>
         <v/>
@@ -16995,7 +17011,7 @@
         <v/>
       </c>
     </row>
-    <row r="252" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="252" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A252" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A252="","",'Carga Vigilador'!A252)</f>
         <v/>
@@ -17035,7 +17051,7 @@
         <v/>
       </c>
     </row>
-    <row r="253" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="253" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A253" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A253="","",'Carga Vigilador'!A253)</f>
         <v/>
@@ -17075,7 +17091,7 @@
         <v/>
       </c>
     </row>
-    <row r="254" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="254" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A254" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A254="","",'Carga Vigilador'!A254)</f>
         <v/>
@@ -17115,7 +17131,7 @@
         <v/>
       </c>
     </row>
-    <row r="255" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="255" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A255" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A255="","",'Carga Vigilador'!A255)</f>
         <v/>
@@ -17155,7 +17171,7 @@
         <v/>
       </c>
     </row>
-    <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="256" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A256" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A256="","",'Carga Vigilador'!A256)</f>
         <v/>
@@ -17195,7 +17211,7 @@
         <v/>
       </c>
     </row>
-    <row r="257" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="257" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A257" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A257="","",'Carga Vigilador'!A257)</f>
         <v/>
@@ -17235,7 +17251,7 @@
         <v/>
       </c>
     </row>
-    <row r="258" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="258" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A258" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A258="","",'Carga Vigilador'!A258)</f>
         <v/>
@@ -17275,7 +17291,7 @@
         <v/>
       </c>
     </row>
-    <row r="259" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="259" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A259" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A259="","",'Carga Vigilador'!A259)</f>
         <v/>
@@ -17315,7 +17331,7 @@
         <v/>
       </c>
     </row>
-    <row r="260" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="260" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A260" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A260="","",'Carga Vigilador'!A260)</f>
         <v/>
@@ -17355,7 +17371,7 @@
         <v/>
       </c>
     </row>
-    <row r="261" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="261" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A261" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A261="","",'Carga Vigilador'!A261)</f>
         <v/>
@@ -17395,7 +17411,7 @@
         <v/>
       </c>
     </row>
-    <row r="262" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="262" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A262" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A262="","",'Carga Vigilador'!A262)</f>
         <v/>
@@ -17435,7 +17451,7 @@
         <v/>
       </c>
     </row>
-    <row r="263" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="263" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A263" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A263="","",'Carga Vigilador'!A263)</f>
         <v/>
@@ -17475,7 +17491,7 @@
         <v/>
       </c>
     </row>
-    <row r="264" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="264" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A264" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A264="","",'Carga Vigilador'!A264)</f>
         <v/>
@@ -17515,7 +17531,7 @@
         <v/>
       </c>
     </row>
-    <row r="265" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="265" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A265" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A265="","",'Carga Vigilador'!A265)</f>
         <v/>
@@ -17555,7 +17571,7 @@
         <v/>
       </c>
     </row>
-    <row r="266" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="266" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A266" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A266="","",'Carga Vigilador'!A266)</f>
         <v/>
@@ -17595,7 +17611,7 @@
         <v/>
       </c>
     </row>
-    <row r="267" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="267" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A267" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A267="","",'Carga Vigilador'!A267)</f>
         <v/>
@@ -17635,7 +17651,7 @@
         <v/>
       </c>
     </row>
-    <row r="268" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="268" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A268" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A268="","",'Carga Vigilador'!A268)</f>
         <v/>
@@ -17675,7 +17691,7 @@
         <v/>
       </c>
     </row>
-    <row r="269" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="269" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A269" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A269="","",'Carga Vigilador'!A269)</f>
         <v/>
@@ -17715,7 +17731,7 @@
         <v/>
       </c>
     </row>
-    <row r="270" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="270" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A270" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A270="","",'Carga Vigilador'!A270)</f>
         <v/>
@@ -17755,7 +17771,7 @@
         <v/>
       </c>
     </row>
-    <row r="271" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="271" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A271" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A271="","",'Carga Vigilador'!A271)</f>
         <v/>
@@ -17795,7 +17811,7 @@
         <v/>
       </c>
     </row>
-    <row r="272" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="272" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A272" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A272="","",'Carga Vigilador'!A272)</f>
         <v/>
@@ -17835,7 +17851,7 @@
         <v/>
       </c>
     </row>
-    <row r="273" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="273" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A273" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A273="","",'Carga Vigilador'!A273)</f>
         <v/>
@@ -17875,7 +17891,7 @@
         <v/>
       </c>
     </row>
-    <row r="274" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="274" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A274" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A274="","",'Carga Vigilador'!A274)</f>
         <v/>
@@ -17915,7 +17931,7 @@
         <v/>
       </c>
     </row>
-    <row r="275" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="275" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A275" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A275="","",'Carga Vigilador'!A275)</f>
         <v/>
@@ -17955,7 +17971,7 @@
         <v/>
       </c>
     </row>
-    <row r="276" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="276" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A276" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A276="","",'Carga Vigilador'!A276)</f>
         <v/>
@@ -17995,7 +18011,7 @@
         <v/>
       </c>
     </row>
-    <row r="277" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="277" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A277" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A277="","",'Carga Vigilador'!A277)</f>
         <v/>
@@ -18035,7 +18051,7 @@
         <v/>
       </c>
     </row>
-    <row r="278" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="278" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A278" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A278="","",'Carga Vigilador'!A278)</f>
         <v/>
@@ -18075,7 +18091,7 @@
         <v/>
       </c>
     </row>
-    <row r="279" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="279" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A279" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A279="","",'Carga Vigilador'!A279)</f>
         <v/>
@@ -18115,7 +18131,7 @@
         <v/>
       </c>
     </row>
-    <row r="280" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="280" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A280" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A280="","",'Carga Vigilador'!A280)</f>
         <v/>
@@ -18155,7 +18171,7 @@
         <v/>
       </c>
     </row>
-    <row r="281" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="281" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A281" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A281="","",'Carga Vigilador'!A281)</f>
         <v/>
@@ -18195,7 +18211,7 @@
         <v/>
       </c>
     </row>
-    <row r="282" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="282" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A282" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A282="","",'Carga Vigilador'!A282)</f>
         <v/>
@@ -18235,7 +18251,7 @@
         <v/>
       </c>
     </row>
-    <row r="283" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="283" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A283" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A283="","",'Carga Vigilador'!A283)</f>
         <v/>
@@ -18275,7 +18291,7 @@
         <v/>
       </c>
     </row>
-    <row r="284" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="284" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A284" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A284="","",'Carga Vigilador'!A284)</f>
         <v/>
@@ -18315,7 +18331,7 @@
         <v/>
       </c>
     </row>
-    <row r="285" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="285" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A285" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A285="","",'Carga Vigilador'!A285)</f>
         <v/>
@@ -18355,7 +18371,7 @@
         <v/>
       </c>
     </row>
-    <row r="286" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="286" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A286" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A286="","",'Carga Vigilador'!A286)</f>
         <v/>
@@ -18395,7 +18411,7 @@
         <v/>
       </c>
     </row>
-    <row r="287" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="287" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A287" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A287="","",'Carga Vigilador'!A287)</f>
         <v/>
@@ -18435,7 +18451,7 @@
         <v/>
       </c>
     </row>
-    <row r="288" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="288" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A288" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A288="","",'Carga Vigilador'!A288)</f>
         <v/>
@@ -18475,7 +18491,7 @@
         <v/>
       </c>
     </row>
-    <row r="289" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="289" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A289" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A289="","",'Carga Vigilador'!A289)</f>
         <v/>
@@ -18515,7 +18531,7 @@
         <v/>
       </c>
     </row>
-    <row r="290" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="290" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A290" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A290="","",'Carga Vigilador'!A290)</f>
         <v/>
@@ -18555,7 +18571,7 @@
         <v/>
       </c>
     </row>
-    <row r="291" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="291" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A291" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A291="","",'Carga Vigilador'!A291)</f>
         <v/>
@@ -18595,7 +18611,7 @@
         <v/>
       </c>
     </row>
-    <row r="292" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="292" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A292" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A292="","",'Carga Vigilador'!A292)</f>
         <v/>
@@ -18635,7 +18651,7 @@
         <v/>
       </c>
     </row>
-    <row r="293" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="293" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A293" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A293="","",'Carga Vigilador'!A293)</f>
         <v/>
@@ -18675,7 +18691,7 @@
         <v/>
       </c>
     </row>
-    <row r="294" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="294" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A294" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A294="","",'Carga Vigilador'!A294)</f>
         <v/>
@@ -18715,7 +18731,7 @@
         <v/>
       </c>
     </row>
-    <row r="295" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="295" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A295" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A295="","",'Carga Vigilador'!A295)</f>
         <v/>
@@ -18755,7 +18771,7 @@
         <v/>
       </c>
     </row>
-    <row r="296" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="296" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A296" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A296="","",'Carga Vigilador'!A296)</f>
         <v/>
@@ -18795,7 +18811,7 @@
         <v/>
       </c>
     </row>
-    <row r="297" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="297" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A297" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A297="","",'Carga Vigilador'!A297)</f>
         <v/>
@@ -18835,7 +18851,7 @@
         <v/>
       </c>
     </row>
-    <row r="298" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="298" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A298" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A298="","",'Carga Vigilador'!A298)</f>
         <v/>
@@ -18875,7 +18891,7 @@
         <v/>
       </c>
     </row>
-    <row r="299" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="299" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A299" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A299="","",'Carga Vigilador'!A299)</f>
         <v/>
@@ -18915,7 +18931,7 @@
         <v/>
       </c>
     </row>
-    <row r="300" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="300" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A300" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A300="","",'Carga Vigilador'!A300)</f>
         <v/>
@@ -18955,7 +18971,7 @@
         <v/>
       </c>
     </row>
-    <row r="301" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="301" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A301" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A301="","",'Carga Vigilador'!A301)</f>
         <v/>
@@ -18995,7 +19011,7 @@
         <v/>
       </c>
     </row>
-    <row r="302" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="302" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A302" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A302="","",'Carga Vigilador'!A302)</f>
         <v/>
@@ -19035,7 +19051,7 @@
         <v/>
       </c>
     </row>
-    <row r="303" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="303" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A303" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A303="","",'Carga Vigilador'!A303)</f>
         <v/>
@@ -19075,7 +19091,7 @@
         <v/>
       </c>
     </row>
-    <row r="304" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="304" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A304" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A304="","",'Carga Vigilador'!A304)</f>
         <v/>
@@ -19115,7 +19131,7 @@
         <v/>
       </c>
     </row>
-    <row r="305" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="305" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A305" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A305="","",'Carga Vigilador'!A305)</f>
         <v/>
@@ -19155,7 +19171,7 @@
         <v/>
       </c>
     </row>
-    <row r="306" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="306" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A306" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A306="","",'Carga Vigilador'!A306)</f>
         <v/>
@@ -19195,7 +19211,7 @@
         <v/>
       </c>
     </row>
-    <row r="307" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="307" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A307" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A307="","",'Carga Vigilador'!A307)</f>
         <v/>
@@ -19235,7 +19251,7 @@
         <v/>
       </c>
     </row>
-    <row r="308" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="308" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A308" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A308="","",'Carga Vigilador'!A308)</f>
         <v/>
@@ -19275,7 +19291,7 @@
         <v/>
       </c>
     </row>
-    <row r="309" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="309" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A309" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A309="","",'Carga Vigilador'!A309)</f>
         <v/>
@@ -19315,7 +19331,7 @@
         <v/>
       </c>
     </row>
-    <row r="310" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="310" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A310" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A310="","",'Carga Vigilador'!A310)</f>
         <v/>
@@ -19355,7 +19371,7 @@
         <v/>
       </c>
     </row>
-    <row r="311" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="311" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A311" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A311="","",'Carga Vigilador'!A311)</f>
         <v/>
@@ -19395,7 +19411,7 @@
         <v/>
       </c>
     </row>
-    <row r="312" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="312" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A312" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A312="","",'Carga Vigilador'!A312)</f>
         <v/>
@@ -19435,7 +19451,7 @@
         <v/>
       </c>
     </row>
-    <row r="313" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="313" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A313" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A313="","",'Carga Vigilador'!A313)</f>
         <v/>
@@ -19475,7 +19491,7 @@
         <v/>
       </c>
     </row>
-    <row r="314" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="314" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A314" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A314="","",'Carga Vigilador'!A314)</f>
         <v/>
@@ -19515,7 +19531,7 @@
         <v/>
       </c>
     </row>
-    <row r="315" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="315" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A315" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A315="","",'Carga Vigilador'!A315)</f>
         <v/>
@@ -19555,7 +19571,7 @@
         <v/>
       </c>
     </row>
-    <row r="316" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="316" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A316" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A316="","",'Carga Vigilador'!A316)</f>
         <v/>
@@ -19595,7 +19611,7 @@
         <v/>
       </c>
     </row>
-    <row r="317" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="317" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A317" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A317="","",'Carga Vigilador'!A317)</f>
         <v/>
@@ -19635,7 +19651,7 @@
         <v/>
       </c>
     </row>
-    <row r="318" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="318" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A318" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A318="","",'Carga Vigilador'!A318)</f>
         <v/>
@@ -19675,7 +19691,7 @@
         <v/>
       </c>
     </row>
-    <row r="319" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="319" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A319" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A319="","",'Carga Vigilador'!A319)</f>
         <v/>
@@ -19715,7 +19731,7 @@
         <v/>
       </c>
     </row>
-    <row r="320" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="320" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A320" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A320="","",'Carga Vigilador'!A320)</f>
         <v/>
@@ -19755,7 +19771,7 @@
         <v/>
       </c>
     </row>
-    <row r="321" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="321" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A321" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A321="","",'Carga Vigilador'!A321)</f>
         <v/>
@@ -19795,7 +19811,7 @@
         <v/>
       </c>
     </row>
-    <row r="322" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="322" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A322" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A322="","",'Carga Vigilador'!A322)</f>
         <v/>
@@ -19835,7 +19851,7 @@
         <v/>
       </c>
     </row>
-    <row r="323" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="323" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A323" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A323="","",'Carga Vigilador'!A323)</f>
         <v/>
@@ -19875,7 +19891,7 @@
         <v/>
       </c>
     </row>
-    <row r="324" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="324" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A324" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A324="","",'Carga Vigilador'!A324)</f>
         <v/>
@@ -19915,7 +19931,7 @@
         <v/>
       </c>
     </row>
-    <row r="325" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="325" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A325" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A325="","",'Carga Vigilador'!A325)</f>
         <v/>
@@ -19955,7 +19971,7 @@
         <v/>
       </c>
     </row>
-    <row r="326" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="326" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A326" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A326="","",'Carga Vigilador'!A326)</f>
         <v/>
@@ -19995,7 +20011,7 @@
         <v/>
       </c>
     </row>
-    <row r="327" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="327" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A327" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A327="","",'Carga Vigilador'!A327)</f>
         <v/>
@@ -20035,7 +20051,7 @@
         <v/>
       </c>
     </row>
-    <row r="328" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="328" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A328" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A328="","",'Carga Vigilador'!A328)</f>
         <v/>
@@ -20075,7 +20091,7 @@
         <v/>
       </c>
     </row>
-    <row r="329" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="329" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A329" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A329="","",'Carga Vigilador'!A329)</f>
         <v/>
@@ -20115,7 +20131,7 @@
         <v/>
       </c>
     </row>
-    <row r="330" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="330" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A330" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A330="","",'Carga Vigilador'!A330)</f>
         <v/>
@@ -20155,7 +20171,7 @@
         <v/>
       </c>
     </row>
-    <row r="331" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="331" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A331" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A331="","",'Carga Vigilador'!A331)</f>
         <v/>
@@ -20195,7 +20211,7 @@
         <v/>
       </c>
     </row>
-    <row r="332" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="332" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A332" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A332="","",'Carga Vigilador'!A332)</f>
         <v/>
@@ -20235,7 +20251,7 @@
         <v/>
       </c>
     </row>
-    <row r="333" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="333" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A333" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A333="","",'Carga Vigilador'!A333)</f>
         <v/>
@@ -20275,7 +20291,7 @@
         <v/>
       </c>
     </row>
-    <row r="334" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="334" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A334" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A334="","",'Carga Vigilador'!A334)</f>
         <v/>
@@ -20315,7 +20331,7 @@
         <v/>
       </c>
     </row>
-    <row r="335" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="335" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A335" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A335="","",'Carga Vigilador'!A335)</f>
         <v/>
@@ -20355,7 +20371,7 @@
         <v/>
       </c>
     </row>
-    <row r="336" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="336" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A336" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A336="","",'Carga Vigilador'!A336)</f>
         <v/>
@@ -20395,7 +20411,7 @@
         <v/>
       </c>
     </row>
-    <row r="337" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="337" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A337" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A337="","",'Carga Vigilador'!A337)</f>
         <v/>
@@ -20435,7 +20451,7 @@
         <v/>
       </c>
     </row>
-    <row r="338" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="338" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A338" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A338="","",'Carga Vigilador'!A338)</f>
         <v/>
@@ -20475,7 +20491,7 @@
         <v/>
       </c>
     </row>
-    <row r="339" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="339" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A339" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A339="","",'Carga Vigilador'!A339)</f>
         <v/>
@@ -20515,7 +20531,7 @@
         <v/>
       </c>
     </row>
-    <row r="340" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="340" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A340" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A340="","",'Carga Vigilador'!A340)</f>
         <v/>
@@ -20555,7 +20571,7 @@
         <v/>
       </c>
     </row>
-    <row r="341" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="341" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A341" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A341="","",'Carga Vigilador'!A341)</f>
         <v/>
@@ -20595,7 +20611,7 @@
         <v/>
       </c>
     </row>
-    <row r="342" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="342" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A342" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A342="","",'Carga Vigilador'!A342)</f>
         <v/>
@@ -20635,7 +20651,7 @@
         <v/>
       </c>
     </row>
-    <row r="343" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="343" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A343" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A343="","",'Carga Vigilador'!A343)</f>
         <v/>
@@ -20675,7 +20691,7 @@
         <v/>
       </c>
     </row>
-    <row r="344" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="344" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A344" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A344="","",'Carga Vigilador'!A344)</f>
         <v/>
@@ -20715,7 +20731,7 @@
         <v/>
       </c>
     </row>
-    <row r="345" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="345" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A345" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A345="","",'Carga Vigilador'!A345)</f>
         <v/>
@@ -20755,7 +20771,7 @@
         <v/>
       </c>
     </row>
-    <row r="346" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="346" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A346" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A346="","",'Carga Vigilador'!A346)</f>
         <v/>
@@ -20795,7 +20811,7 @@
         <v/>
       </c>
     </row>
-    <row r="347" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="347" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A347" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A347="","",'Carga Vigilador'!A347)</f>
         <v/>
@@ -20835,7 +20851,7 @@
         <v/>
       </c>
     </row>
-    <row r="348" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="348" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A348" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A348="","",'Carga Vigilador'!A348)</f>
         <v/>
@@ -20875,7 +20891,7 @@
         <v/>
       </c>
     </row>
-    <row r="349" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="349" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A349" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A349="","",'Carga Vigilador'!A349)</f>
         <v/>
@@ -20915,7 +20931,7 @@
         <v/>
       </c>
     </row>
-    <row r="350" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="350" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A350" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A350="","",'Carga Vigilador'!A350)</f>
         <v/>
@@ -20955,7 +20971,7 @@
         <v/>
       </c>
     </row>
-    <row r="351" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="351" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A351" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A351="","",'Carga Vigilador'!A351)</f>
         <v/>
@@ -20995,7 +21011,7 @@
         <v/>
       </c>
     </row>
-    <row r="352" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="352" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A352" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A352="","",'Carga Vigilador'!A352)</f>
         <v/>
@@ -21035,7 +21051,7 @@
         <v/>
       </c>
     </row>
-    <row r="353" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="353" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A353" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A353="","",'Carga Vigilador'!A353)</f>
         <v/>
@@ -21075,7 +21091,7 @@
         <v/>
       </c>
     </row>
-    <row r="354" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="354" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A354" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A354="","",'Carga Vigilador'!A354)</f>
         <v/>
@@ -21115,7 +21131,7 @@
         <v/>
       </c>
     </row>
-    <row r="355" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="355" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A355" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A355="","",'Carga Vigilador'!A355)</f>
         <v/>
@@ -21155,7 +21171,7 @@
         <v/>
       </c>
     </row>
-    <row r="356" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="356" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A356" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A356="","",'Carga Vigilador'!A356)</f>
         <v/>
@@ -21195,7 +21211,7 @@
         <v/>
       </c>
     </row>
-    <row r="357" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="357" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A357" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A357="","",'Carga Vigilador'!A357)</f>
         <v/>
@@ -21235,7 +21251,7 @@
         <v/>
       </c>
     </row>
-    <row r="358" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="358" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A358" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A358="","",'Carga Vigilador'!A358)</f>
         <v/>
@@ -21275,7 +21291,7 @@
         <v/>
       </c>
     </row>
-    <row r="359" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="359" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A359" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A359="","",'Carga Vigilador'!A359)</f>
         <v/>
@@ -21315,7 +21331,7 @@
         <v/>
       </c>
     </row>
-    <row r="360" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="360" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A360" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A360="","",'Carga Vigilador'!A360)</f>
         <v/>
@@ -21355,7 +21371,7 @@
         <v/>
       </c>
     </row>
-    <row r="361" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="361" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A361" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A361="","",'Carga Vigilador'!A361)</f>
         <v/>
@@ -21395,7 +21411,7 @@
         <v/>
       </c>
     </row>
-    <row r="362" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="362" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A362" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A362="","",'Carga Vigilador'!A362)</f>
         <v/>
@@ -21435,7 +21451,7 @@
         <v/>
       </c>
     </row>
-    <row r="363" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="363" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A363" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A363="","",'Carga Vigilador'!A363)</f>
         <v/>
@@ -21475,7 +21491,7 @@
         <v/>
       </c>
     </row>
-    <row r="364" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="364" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A364" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A364="","",'Carga Vigilador'!A364)</f>
         <v/>
@@ -21515,7 +21531,7 @@
         <v/>
       </c>
     </row>
-    <row r="365" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="365" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A365" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A365="","",'Carga Vigilador'!A365)</f>
         <v/>
@@ -21555,7 +21571,7 @@
         <v/>
       </c>
     </row>
-    <row r="366" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="366" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A366" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A366="","",'Carga Vigilador'!A366)</f>
         <v/>
@@ -21595,7 +21611,7 @@
         <v/>
       </c>
     </row>
-    <row r="367" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="367" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A367" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A367="","",'Carga Vigilador'!A367)</f>
         <v/>
@@ -21635,7 +21651,7 @@
         <v/>
       </c>
     </row>
-    <row r="368" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="368" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A368" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A368="","",'Carga Vigilador'!A368)</f>
         <v/>
@@ -21675,7 +21691,7 @@
         <v/>
       </c>
     </row>
-    <row r="369" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="369" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A369" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A369="","",'Carga Vigilador'!A369)</f>
         <v/>
@@ -21715,7 +21731,7 @@
         <v/>
       </c>
     </row>
-    <row r="370" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="370" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A370" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A370="","",'Carga Vigilador'!A370)</f>
         <v/>
@@ -21755,7 +21771,7 @@
         <v/>
       </c>
     </row>
-    <row r="371" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="371" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A371" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A371="","",'Carga Vigilador'!A371)</f>
         <v/>
@@ -21795,7 +21811,7 @@
         <v/>
       </c>
     </row>
-    <row r="372" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="372" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A372" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A372="","",'Carga Vigilador'!A372)</f>
         <v/>
@@ -21835,7 +21851,7 @@
         <v/>
       </c>
     </row>
-    <row r="373" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="373" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A373" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A373="","",'Carga Vigilador'!A373)</f>
         <v/>
@@ -21875,7 +21891,7 @@
         <v/>
       </c>
     </row>
-    <row r="374" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="374" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A374" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A374="","",'Carga Vigilador'!A374)</f>
         <v/>
@@ -21915,7 +21931,7 @@
         <v/>
       </c>
     </row>
-    <row r="375" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="375" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A375" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A375="","",'Carga Vigilador'!A375)</f>
         <v/>
@@ -21955,7 +21971,7 @@
         <v/>
       </c>
     </row>
-    <row r="376" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="376" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A376" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A376="","",'Carga Vigilador'!A376)</f>
         <v/>
@@ -21995,7 +22011,7 @@
         <v/>
       </c>
     </row>
-    <row r="377" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="377" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A377" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A377="","",'Carga Vigilador'!A377)</f>
         <v/>
@@ -22035,7 +22051,7 @@
         <v/>
       </c>
     </row>
-    <row r="378" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="378" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A378" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A378="","",'Carga Vigilador'!A378)</f>
         <v/>
@@ -22075,7 +22091,7 @@
         <v/>
       </c>
     </row>
-    <row r="379" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="379" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A379" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A379="","",'Carga Vigilador'!A379)</f>
         <v/>
@@ -22115,7 +22131,7 @@
         <v/>
       </c>
     </row>
-    <row r="380" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="380" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A380" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A380="","",'Carga Vigilador'!A380)</f>
         <v/>
@@ -22155,7 +22171,7 @@
         <v/>
       </c>
     </row>
-    <row r="381" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="381" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A381" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A381="","",'Carga Vigilador'!A381)</f>
         <v/>
@@ -22195,7 +22211,7 @@
         <v/>
       </c>
     </row>
-    <row r="382" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="382" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A382" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A382="","",'Carga Vigilador'!A382)</f>
         <v/>
@@ -22235,7 +22251,7 @@
         <v/>
       </c>
     </row>
-    <row r="383" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="383" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A383" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A383="","",'Carga Vigilador'!A383)</f>
         <v/>
@@ -22275,7 +22291,7 @@
         <v/>
       </c>
     </row>
-    <row r="384" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="384" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A384" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A384="","",'Carga Vigilador'!A384)</f>
         <v/>
@@ -22315,7 +22331,7 @@
         <v/>
       </c>
     </row>
-    <row r="385" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="385" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A385" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A385="","",'Carga Vigilador'!A385)</f>
         <v/>
@@ -22355,7 +22371,7 @@
         <v/>
       </c>
     </row>
-    <row r="386" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="386" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A386" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A386="","",'Carga Vigilador'!A386)</f>
         <v/>
@@ -22395,7 +22411,7 @@
         <v/>
       </c>
     </row>
-    <row r="387" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="387" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A387" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A387="","",'Carga Vigilador'!A387)</f>
         <v/>
@@ -22435,7 +22451,7 @@
         <v/>
       </c>
     </row>
-    <row r="388" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="388" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A388" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A388="","",'Carga Vigilador'!A388)</f>
         <v/>
@@ -22475,7 +22491,7 @@
         <v/>
       </c>
     </row>
-    <row r="389" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="389" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A389" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A389="","",'Carga Vigilador'!A389)</f>
         <v/>
@@ -22515,7 +22531,7 @@
         <v/>
       </c>
     </row>
-    <row r="390" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="390" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A390" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A390="","",'Carga Vigilador'!A390)</f>
         <v/>
@@ -22555,7 +22571,7 @@
         <v/>
       </c>
     </row>
-    <row r="391" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="391" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A391" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A391="","",'Carga Vigilador'!A391)</f>
         <v/>
@@ -22595,7 +22611,7 @@
         <v/>
       </c>
     </row>
-    <row r="392" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="392" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A392" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A392="","",'Carga Vigilador'!A392)</f>
         <v/>
@@ -22635,7 +22651,7 @@
         <v/>
       </c>
     </row>
-    <row r="393" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="393" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A393" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A393="","",'Carga Vigilador'!A393)</f>
         <v/>
@@ -22675,7 +22691,7 @@
         <v/>
       </c>
     </row>
-    <row r="394" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="394" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A394" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A394="","",'Carga Vigilador'!A394)</f>
         <v/>
@@ -22715,7 +22731,7 @@
         <v/>
       </c>
     </row>
-    <row r="395" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="395" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A395" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A395="","",'Carga Vigilador'!A395)</f>
         <v/>
@@ -22755,7 +22771,7 @@
         <v/>
       </c>
     </row>
-    <row r="396" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="396" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A396" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A396="","",'Carga Vigilador'!A396)</f>
         <v/>
@@ -22795,7 +22811,7 @@
         <v/>
       </c>
     </row>
-    <row r="397" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="397" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A397" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A397="","",'Carga Vigilador'!A397)</f>
         <v/>
@@ -22835,7 +22851,7 @@
         <v/>
       </c>
     </row>
-    <row r="398" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="398" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A398" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A398="","",'Carga Vigilador'!A398)</f>
         <v/>
@@ -22875,7 +22891,7 @@
         <v/>
       </c>
     </row>
-    <row r="399" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="399" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A399" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A399="","",'Carga Vigilador'!A399)</f>
         <v/>
@@ -22915,7 +22931,7 @@
         <v/>
       </c>
     </row>
-    <row r="400" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="400" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A400" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A400="","",'Carga Vigilador'!A400)</f>
         <v/>
@@ -22955,7 +22971,7 @@
         <v/>
       </c>
     </row>
-    <row r="401" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="401" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A401" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A401="","",'Carga Vigilador'!A401)</f>
         <v/>
@@ -22995,7 +23011,7 @@
         <v/>
       </c>
     </row>
-    <row r="402" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="402" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A402" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A402="","",'Carga Vigilador'!A402)</f>
         <v/>
@@ -23035,7 +23051,7 @@
         <v/>
       </c>
     </row>
-    <row r="403" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="403" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A403" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A403="","",'Carga Vigilador'!A403)</f>
         <v/>
@@ -23075,7 +23091,7 @@
         <v/>
       </c>
     </row>
-    <row r="404" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="404" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A404" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A404="","",'Carga Vigilador'!A404)</f>
         <v/>
@@ -23115,7 +23131,7 @@
         <v/>
       </c>
     </row>
-    <row r="405" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="405" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A405" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A405="","",'Carga Vigilador'!A405)</f>
         <v/>
@@ -23155,7 +23171,7 @@
         <v/>
       </c>
     </row>
-    <row r="406" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="406" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A406" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A406="","",'Carga Vigilador'!A406)</f>
         <v/>
@@ -23195,7 +23211,7 @@
         <v/>
       </c>
     </row>
-    <row r="407" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="407" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A407" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A407="","",'Carga Vigilador'!A407)</f>
         <v/>
@@ -23235,7 +23251,7 @@
         <v/>
       </c>
     </row>
-    <row r="408" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="408" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A408" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A408="","",'Carga Vigilador'!A408)</f>
         <v/>
@@ -23275,7 +23291,7 @@
         <v/>
       </c>
     </row>
-    <row r="409" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="409" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A409" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A409="","",'Carga Vigilador'!A409)</f>
         <v/>
@@ -23315,7 +23331,7 @@
         <v/>
       </c>
     </row>
-    <row r="410" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="410" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A410" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A410="","",'Carga Vigilador'!A410)</f>
         <v/>
@@ -23355,7 +23371,7 @@
         <v/>
       </c>
     </row>
-    <row r="411" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="411" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A411" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A411="","",'Carga Vigilador'!A411)</f>
         <v/>
@@ -23395,7 +23411,7 @@
         <v/>
       </c>
     </row>
-    <row r="412" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="412" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A412" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A412="","",'Carga Vigilador'!A412)</f>
         <v/>
@@ -23435,7 +23451,7 @@
         <v/>
       </c>
     </row>
-    <row r="413" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="413" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A413" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A413="","",'Carga Vigilador'!A413)</f>
         <v/>
@@ -23475,7 +23491,7 @@
         <v/>
       </c>
     </row>
-    <row r="414" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="414" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A414" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A414="","",'Carga Vigilador'!A414)</f>
         <v/>
@@ -23515,7 +23531,7 @@
         <v/>
       </c>
     </row>
-    <row r="415" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="415" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A415" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A415="","",'Carga Vigilador'!A415)</f>
         <v/>
@@ -23555,7 +23571,7 @@
         <v/>
       </c>
     </row>
-    <row r="416" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="416" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A416" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A416="","",'Carga Vigilador'!A416)</f>
         <v/>
@@ -23595,7 +23611,7 @@
         <v/>
       </c>
     </row>
-    <row r="417" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="417" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A417" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A417="","",'Carga Vigilador'!A417)</f>
         <v/>
@@ -23635,7 +23651,7 @@
         <v/>
       </c>
     </row>
-    <row r="418" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="418" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A418" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A418="","",'Carga Vigilador'!A418)</f>
         <v/>
@@ -23675,7 +23691,7 @@
         <v/>
       </c>
     </row>
-    <row r="419" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="419" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A419" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A419="","",'Carga Vigilador'!A419)</f>
         <v/>
@@ -23715,7 +23731,7 @@
         <v/>
       </c>
     </row>
-    <row r="420" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="420" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A420" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A420="","",'Carga Vigilador'!A420)</f>
         <v/>
@@ -23755,7 +23771,7 @@
         <v/>
       </c>
     </row>
-    <row r="421" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="421" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A421" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A421="","",'Carga Vigilador'!A421)</f>
         <v/>
@@ -23795,7 +23811,7 @@
         <v/>
       </c>
     </row>
-    <row r="422" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="422" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A422" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A422="","",'Carga Vigilador'!A422)</f>
         <v/>
@@ -23835,7 +23851,7 @@
         <v/>
       </c>
     </row>
-    <row r="423" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="423" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A423" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A423="","",'Carga Vigilador'!A423)</f>
         <v/>
@@ -23875,7 +23891,7 @@
         <v/>
       </c>
     </row>
-    <row r="424" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="424" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A424" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A424="","",'Carga Vigilador'!A424)</f>
         <v/>
@@ -23915,7 +23931,7 @@
         <v/>
       </c>
     </row>
-    <row r="425" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="425" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A425" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A425="","",'Carga Vigilador'!A425)</f>
         <v/>
@@ -23955,7 +23971,7 @@
         <v/>
       </c>
     </row>
-    <row r="426" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="426" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A426" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A426="","",'Carga Vigilador'!A426)</f>
         <v/>
@@ -23995,7 +24011,7 @@
         <v/>
       </c>
     </row>
-    <row r="427" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="427" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A427" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A427="","",'Carga Vigilador'!A427)</f>
         <v/>
@@ -24035,7 +24051,7 @@
         <v/>
       </c>
     </row>
-    <row r="428" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="428" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A428" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A428="","",'Carga Vigilador'!A428)</f>
         <v/>
@@ -24075,7 +24091,7 @@
         <v/>
       </c>
     </row>
-    <row r="429" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="429" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A429" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A429="","",'Carga Vigilador'!A429)</f>
         <v/>
@@ -24115,7 +24131,7 @@
         <v/>
       </c>
     </row>
-    <row r="430" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="430" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A430" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A430="","",'Carga Vigilador'!A430)</f>
         <v/>
@@ -24155,7 +24171,7 @@
         <v/>
       </c>
     </row>
-    <row r="431" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="431" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A431" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A431="","",'Carga Vigilador'!A431)</f>
         <v/>
@@ -24195,7 +24211,7 @@
         <v/>
       </c>
     </row>
-    <row r="432" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="432" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A432" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A432="","",'Carga Vigilador'!A432)</f>
         <v/>
@@ -24235,7 +24251,7 @@
         <v/>
       </c>
     </row>
-    <row r="433" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="433" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A433" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A433="","",'Carga Vigilador'!A433)</f>
         <v/>
@@ -24275,7 +24291,7 @@
         <v/>
       </c>
     </row>
-    <row r="434" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="434" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A434" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A434="","",'Carga Vigilador'!A434)</f>
         <v/>
@@ -24315,7 +24331,7 @@
         <v/>
       </c>
     </row>
-    <row r="435" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="435" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A435" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A435="","",'Carga Vigilador'!A435)</f>
         <v/>
@@ -24355,7 +24371,7 @@
         <v/>
       </c>
     </row>
-    <row r="436" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="436" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A436" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A436="","",'Carga Vigilador'!A436)</f>
         <v/>
@@ -24395,7 +24411,7 @@
         <v/>
       </c>
     </row>
-    <row r="437" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="437" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A437" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A437="","",'Carga Vigilador'!A437)</f>
         <v/>
@@ -24435,7 +24451,7 @@
         <v/>
       </c>
     </row>
-    <row r="438" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="438" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A438" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A438="","",'Carga Vigilador'!A438)</f>
         <v/>
@@ -24475,7 +24491,7 @@
         <v/>
       </c>
     </row>
-    <row r="439" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="439" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A439" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A439="","",'Carga Vigilador'!A439)</f>
         <v/>
@@ -24515,7 +24531,7 @@
         <v/>
       </c>
     </row>
-    <row r="440" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="440" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A440" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A440="","",'Carga Vigilador'!A440)</f>
         <v/>
@@ -24555,7 +24571,7 @@
         <v/>
       </c>
     </row>
-    <row r="441" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="441" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A441" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A441="","",'Carga Vigilador'!A441)</f>
         <v/>
@@ -24595,7 +24611,7 @@
         <v/>
       </c>
     </row>
-    <row r="442" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="442" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A442" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A442="","",'Carga Vigilador'!A442)</f>
         <v/>
@@ -24635,7 +24651,7 @@
         <v/>
       </c>
     </row>
-    <row r="443" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="443" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A443" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A443="","",'Carga Vigilador'!A443)</f>
         <v/>
@@ -24675,7 +24691,7 @@
         <v/>
       </c>
     </row>
-    <row r="444" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="444" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A444" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A444="","",'Carga Vigilador'!A444)</f>
         <v/>
@@ -24715,7 +24731,7 @@
         <v/>
       </c>
     </row>
-    <row r="445" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="445" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A445" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A445="","",'Carga Vigilador'!A445)</f>
         <v/>
@@ -24755,7 +24771,7 @@
         <v/>
       </c>
     </row>
-    <row r="446" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="446" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A446" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A446="","",'Carga Vigilador'!A446)</f>
         <v/>
@@ -24795,7 +24811,7 @@
         <v/>
       </c>
     </row>
-    <row r="447" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="447" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A447" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A447="","",'Carga Vigilador'!A447)</f>
         <v/>
@@ -24835,7 +24851,7 @@
         <v/>
       </c>
     </row>
-    <row r="448" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="448" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A448" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A448="","",'Carga Vigilador'!A448)</f>
         <v/>
@@ -24875,7 +24891,7 @@
         <v/>
       </c>
     </row>
-    <row r="449" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="449" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A449" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A449="","",'Carga Vigilador'!A449)</f>
         <v/>
@@ -24915,7 +24931,7 @@
         <v/>
       </c>
     </row>
-    <row r="450" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="450" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A450" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A450="","",'Carga Vigilador'!A450)</f>
         <v/>
@@ -24955,7 +24971,7 @@
         <v/>
       </c>
     </row>
-    <row r="451" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="451" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A451" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A451="","",'Carga Vigilador'!A451)</f>
         <v/>
@@ -24995,7 +25011,7 @@
         <v/>
       </c>
     </row>
-    <row r="452" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="452" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A452" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A452="","",'Carga Vigilador'!A452)</f>
         <v/>
@@ -25035,7 +25051,7 @@
         <v/>
       </c>
     </row>
-    <row r="453" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="453" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A453" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A453="","",'Carga Vigilador'!A453)</f>
         <v/>
@@ -25075,7 +25091,7 @@
         <v/>
       </c>
     </row>
-    <row r="454" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="454" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A454" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A454="","",'Carga Vigilador'!A454)</f>
         <v/>
@@ -25115,7 +25131,7 @@
         <v/>
       </c>
     </row>
-    <row r="455" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="455" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A455" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A455="","",'Carga Vigilador'!A455)</f>
         <v/>
@@ -25155,7 +25171,7 @@
         <v/>
       </c>
     </row>
-    <row r="456" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="456" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A456" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A456="","",'Carga Vigilador'!A456)</f>
         <v/>
@@ -25195,7 +25211,7 @@
         <v/>
       </c>
     </row>
-    <row r="457" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="457" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A457" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A457="","",'Carga Vigilador'!A457)</f>
         <v/>
@@ -25235,7 +25251,7 @@
         <v/>
       </c>
     </row>
-    <row r="458" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="458" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A458" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A458="","",'Carga Vigilador'!A458)</f>
         <v/>
@@ -25275,7 +25291,7 @@
         <v/>
       </c>
     </row>
-    <row r="459" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="459" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A459" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A459="","",'Carga Vigilador'!A459)</f>
         <v/>
@@ -25315,7 +25331,7 @@
         <v/>
       </c>
     </row>
-    <row r="460" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="460" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A460" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A460="","",'Carga Vigilador'!A460)</f>
         <v/>
@@ -25355,7 +25371,7 @@
         <v/>
       </c>
     </row>
-    <row r="461" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="461" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A461" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A461="","",'Carga Vigilador'!A461)</f>
         <v/>
@@ -25395,7 +25411,7 @@
         <v/>
       </c>
     </row>
-    <row r="462" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="462" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A462" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A462="","",'Carga Vigilador'!A462)</f>
         <v/>
@@ -25435,7 +25451,7 @@
         <v/>
       </c>
     </row>
-    <row r="463" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="463" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A463" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A463="","",'Carga Vigilador'!A463)</f>
         <v/>
@@ -25475,7 +25491,7 @@
         <v/>
       </c>
     </row>
-    <row r="464" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="464" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A464" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A464="","",'Carga Vigilador'!A464)</f>
         <v/>
@@ -25515,7 +25531,7 @@
         <v/>
       </c>
     </row>
-    <row r="465" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="465" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A465" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A465="","",'Carga Vigilador'!A465)</f>
         <v/>
@@ -25555,7 +25571,7 @@
         <v/>
       </c>
     </row>
-    <row r="466" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="466" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A466" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A466="","",'Carga Vigilador'!A466)</f>
         <v/>
@@ -25595,7 +25611,7 @@
         <v/>
       </c>
     </row>
-    <row r="467" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="467" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A467" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A467="","",'Carga Vigilador'!A467)</f>
         <v/>
@@ -25635,7 +25651,7 @@
         <v/>
       </c>
     </row>
-    <row r="468" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="468" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A468" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A468="","",'Carga Vigilador'!A468)</f>
         <v/>
@@ -25675,7 +25691,7 @@
         <v/>
       </c>
     </row>
-    <row r="469" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="469" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A469" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A469="","",'Carga Vigilador'!A469)</f>
         <v/>
@@ -25715,7 +25731,7 @@
         <v/>
       </c>
     </row>
-    <row r="470" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="470" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A470" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A470="","",'Carga Vigilador'!A470)</f>
         <v/>
@@ -25755,7 +25771,7 @@
         <v/>
       </c>
     </row>
-    <row r="471" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="471" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A471" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A471="","",'Carga Vigilador'!A471)</f>
         <v/>
@@ -25795,7 +25811,7 @@
         <v/>
       </c>
     </row>
-    <row r="472" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="472" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A472" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A472="","",'Carga Vigilador'!A472)</f>
         <v/>
@@ -25835,7 +25851,7 @@
         <v/>
       </c>
     </row>
-    <row r="473" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="473" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A473" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A473="","",'Carga Vigilador'!A473)</f>
         <v/>
@@ -25875,7 +25891,7 @@
         <v/>
       </c>
     </row>
-    <row r="474" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="474" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A474" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A474="","",'Carga Vigilador'!A474)</f>
         <v/>
@@ -25915,7 +25931,7 @@
         <v/>
       </c>
     </row>
-    <row r="475" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="475" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A475" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A475="","",'Carga Vigilador'!A475)</f>
         <v/>
@@ -25955,7 +25971,7 @@
         <v/>
       </c>
     </row>
-    <row r="476" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="476" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A476" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A476="","",'Carga Vigilador'!A476)</f>
         <v/>
@@ -25995,7 +26011,7 @@
         <v/>
       </c>
     </row>
-    <row r="477" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="477" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A477" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A477="","",'Carga Vigilador'!A477)</f>
         <v/>
@@ -26035,7 +26051,7 @@
         <v/>
       </c>
     </row>
-    <row r="478" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="478" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A478" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A478="","",'Carga Vigilador'!A478)</f>
         <v/>
@@ -26075,7 +26091,7 @@
         <v/>
       </c>
     </row>
-    <row r="479" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="479" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A479" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A479="","",'Carga Vigilador'!A479)</f>
         <v/>
@@ -26115,7 +26131,7 @@
         <v/>
       </c>
     </row>
-    <row r="480" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="480" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A480" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A480="","",'Carga Vigilador'!A480)</f>
         <v/>
@@ -26155,7 +26171,7 @@
         <v/>
       </c>
     </row>
-    <row r="481" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="481" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A481" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A481="","",'Carga Vigilador'!A481)</f>
         <v/>
@@ -26195,7 +26211,7 @@
         <v/>
       </c>
     </row>
-    <row r="482" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="482" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A482" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A482="","",'Carga Vigilador'!A482)</f>
         <v/>
@@ -26235,7 +26251,7 @@
         <v/>
       </c>
     </row>
-    <row r="483" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="483" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A483" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A483="","",'Carga Vigilador'!A483)</f>
         <v/>
@@ -26275,7 +26291,7 @@
         <v/>
       </c>
     </row>
-    <row r="484" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="484" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A484" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A484="","",'Carga Vigilador'!A484)</f>
         <v/>
@@ -26315,7 +26331,7 @@
         <v/>
       </c>
     </row>
-    <row r="485" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="485" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A485" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A485="","",'Carga Vigilador'!A485)</f>
         <v/>
@@ -26355,7 +26371,7 @@
         <v/>
       </c>
     </row>
-    <row r="486" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="486" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A486" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A486="","",'Carga Vigilador'!A486)</f>
         <v/>
@@ -26395,7 +26411,7 @@
         <v/>
       </c>
     </row>
-    <row r="487" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="487" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A487" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A487="","",'Carga Vigilador'!A487)</f>
         <v/>
@@ -26435,7 +26451,7 @@
         <v/>
       </c>
     </row>
-    <row r="488" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="488" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A488" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A488="","",'Carga Vigilador'!A488)</f>
         <v/>
@@ -26475,7 +26491,7 @@
         <v/>
       </c>
     </row>
-    <row r="489" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="489" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A489" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A489="","",'Carga Vigilador'!A489)</f>
         <v/>
@@ -26515,7 +26531,7 @@
         <v/>
       </c>
     </row>
-    <row r="490" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="490" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A490" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A490="","",'Carga Vigilador'!A490)</f>
         <v/>
@@ -26555,7 +26571,7 @@
         <v/>
       </c>
     </row>
-    <row r="491" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="491" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A491" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A491="","",'Carga Vigilador'!A491)</f>
         <v/>
@@ -26595,7 +26611,7 @@
         <v/>
       </c>
     </row>
-    <row r="492" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="492" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A492" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A492="","",'Carga Vigilador'!A492)</f>
         <v/>
@@ -26635,7 +26651,7 @@
         <v/>
       </c>
     </row>
-    <row r="493" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="493" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A493" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A493="","",'Carga Vigilador'!A493)</f>
         <v/>
@@ -26675,7 +26691,7 @@
         <v/>
       </c>
     </row>
-    <row r="494" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="494" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A494" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A494="","",'Carga Vigilador'!A494)</f>
         <v/>
@@ -26715,7 +26731,7 @@
         <v/>
       </c>
     </row>
-    <row r="495" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="495" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A495" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A495="","",'Carga Vigilador'!A495)</f>
         <v/>
@@ -26755,7 +26771,7 @@
         <v/>
       </c>
     </row>
-    <row r="496" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="496" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A496" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A496="","",'Carga Vigilador'!A496)</f>
         <v/>
@@ -26795,7 +26811,7 @@
         <v/>
       </c>
     </row>
-    <row r="497" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="497" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A497" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A497="","",'Carga Vigilador'!A497)</f>
         <v/>
@@ -26835,7 +26851,7 @@
         <v/>
       </c>
     </row>
-    <row r="498" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="498" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A498" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A498="","",'Carga Vigilador'!A498)</f>
         <v/>
@@ -26875,7 +26891,7 @@
         <v/>
       </c>
     </row>
-    <row r="499" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="499" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A499" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A499="","",'Carga Vigilador'!A499)</f>
         <v/>
@@ -26915,7 +26931,7 @@
         <v/>
       </c>
     </row>
-    <row r="500" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="500" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A500" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A500="","",'Carga Vigilador'!A500)</f>
         <v/>
@@ -26955,7 +26971,7 @@
         <v/>
       </c>
     </row>
-    <row r="501" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="501" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A501" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A501="","",'Carga Vigilador'!A501)</f>
         <v/>
@@ -26995,7 +27011,7 @@
         <v/>
       </c>
     </row>
-    <row r="502" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="502" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A502" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A502="","",'Carga Vigilador'!A502)</f>
         <v/>
@@ -27035,7 +27051,7 @@
         <v/>
       </c>
     </row>
-    <row r="503" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="503" customFormat="false" ht="90" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A503" s="6" t="str">
         <f aca="false">IF('Carga Vigilador'!A503="","",'Carga Vigilador'!A503)</f>
         <v/>
@@ -27127,17 +27143,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B4" s="20" t="n">
         <v>46296</v>
@@ -27145,7 +27161,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B5" s="20" t="n">
         <v>46326</v>
@@ -27153,82 +27169,82 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B6" s="21"/>
       <c r="C6" s="4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="22" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B9" s="24" t="n">
         <f aca="false">IF($B$6="",COUNTIFS('Carga Administración'!$B$4:$B$503,"&gt;="&amp;$B$4,'Carga Administración'!$B$4:$B$503,"&lt;="&amp;$B$5),COUNTIFS('Carga Administración'!$B$4:$B$503,"&gt;="&amp;$B$4,'Carga Administración'!$B$4:$B$503,"&lt;="&amp;$B$5,'Carga Administración'!$E$4:$E$503,$B$6))</f>
         <v>1</v>
       </c>
       <c r="C9" s="25" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="23" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B10" s="24" t="n">
         <f aca="false">IF($B$6="",COUNTIFS('Carga Administración'!$H$4:$H$503,"Sí",'Carga Administración'!$I$4:$I$503,"&gt;="&amp;$B$4,'Carga Administración'!$I$4:$I$503,"&lt;="&amp;$B$5),COUNTIFS('Carga Administración'!$H$4:$H$503,"Sí",'Carga Administración'!$I$4:$I$503,"&gt;="&amp;$B$4,'Carga Administración'!$I$4:$I$503,"&lt;="&amp;$B$5,'Carga Administración'!$E$4:$E$503,$B$6))</f>
         <v>0</v>
       </c>
       <c r="C10" s="25" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B11" s="24" t="n">
         <f aca="false">IF($B$6="",COUNTIFS('Carga Administración'!$J$4:$J$503,"Sí",'Carga Administración'!$K$4:$K$503,"&gt;="&amp;$B$4,'Carga Administración'!$K$4:$K$503,"&lt;="&amp;$B$5),COUNTIFS('Carga Administración'!$J$4:$J$503,"Sí",'Carga Administración'!$K$4:$K$503,"&gt;="&amp;$B$4,'Carga Administración'!$K$4:$K$503,"&lt;="&amp;$B$5,'Carga Administración'!$E$4:$E$503,$B$6))</f>
         <v>0</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="23" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B12" s="26" t="n">
         <f aca="false">IF($B$6="",SUMIFS('Carga Administración'!$L$4:$L$503,'Carga Administración'!$J$4:$J$503,"Sí",'Carga Administración'!$K$4:$K$503,"&gt;="&amp;$B$4,'Carga Administración'!$K$4:$K$503,"&lt;="&amp;$B$5),SUMIFS('Carga Administración'!$L$4:$L$503,'Carga Administración'!$J$4:$J$503,"Sí",'Carga Administración'!$K$4:$K$503,"&gt;="&amp;$B$4,'Carga Administración'!$K$4:$K$503,"&lt;="&amp;$B$5,'Carga Administración'!$E$4:$E$503,$B$6))</f>
         <v>0</v>
       </c>
       <c r="C12" s="25" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="23" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B13" s="24" t="n">
         <f aca="false">IF($B$6="",COUNTIFS('Carga Administración'!$N$4:$N$503,"Pendiente",'Carga Administración'!$B$4:$B$503,"&gt;="&amp;$B$4,'Carga Administración'!$B$4:$B$503,"&lt;="&amp;$B$5),COUNTIFS('Carga Administración'!$N$4:$N$503,"Pendiente",'Carga Administración'!$B$4:$B$503,"&gt;="&amp;$B$4,'Carga Administración'!$B$4:$B$503,"&lt;="&amp;$B$5,'Carga Administración'!$E$4:$E$503,$B$6))</f>
         <v>1</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>